<commit_message>
streamlining water analysis data
</commit_message>
<xml_diff>
--- a/00_metadata/water_analysis_metadata.xlsx
+++ b/00_metadata/water_analysis_metadata.xlsx
@@ -8,20 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/margaretswift/Documents/03 Science/00 Research - Active/Ecosphere Waterholes/eco-kaza-water-ele/00_metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6A56845-869B-3849-8B81-DC3CC72860B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A75B0D11-77F6-BE42-AD3C-0F91A92B54AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="-7880" windowWidth="20020" windowHeight="21100" activeTab="1" xr2:uid="{36B2674D-5574-5749-ABD1-0B06D0B52360}"/>
+    <workbookView xWindow="29400" yWindow="-7880" windowWidth="20020" windowHeight="21100" activeTab="2" xr2:uid="{36B2674D-5574-5749-ABD1-0B06D0B52360}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
     <sheet name="00_validation.R" sheetId="7" r:id="rId2"/>
+    <sheet name="01_createRasterStats.R" sheetId="8" r:id="rId3"/>
+    <sheet name="02_createPlots.R" sheetId="9" r:id="rId4"/>
+    <sheet name="03_runWaterModels.R" sheetId="10" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="84">
   <si>
     <t>Column Name</t>
   </si>
@@ -35,6 +38,9 @@
     <t>str</t>
   </si>
   <si>
+    <t>mm</t>
+  </si>
+  <si>
     <t>All tables and data exported from the 01_water_analysis set of scripts</t>
   </si>
   <si>
@@ -99,6 +105,177 @@
   </si>
   <si>
     <t>/03_output/Table1.csv</t>
+  </si>
+  <si>
+    <t>Table S4 in Appendix 1 - validation summaries comparing ESW with and without MWF masking</t>
+  </si>
+  <si>
+    <t>ESWNoMWF</t>
+  </si>
+  <si>
+    <t>/03_output/TableS4.csv</t>
+  </si>
+  <si>
+    <t>01_createRasterStats.R</t>
+  </si>
+  <si>
+    <t>Object</t>
+  </si>
+  <si>
+    <t>stats</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>TYPE</t>
+  </si>
+  <si>
+    <t>PERIOD</t>
+  </si>
+  <si>
+    <t>YEAR</t>
+  </si>
+  <si>
+    <t>START</t>
+  </si>
+  <si>
+    <t>END</t>
+  </si>
+  <si>
+    <t>ESW_NPIX</t>
+  </si>
+  <si>
+    <t>MWF_NPIX</t>
+  </si>
+  <si>
+    <t>PX_AREA</t>
+  </si>
+  <si>
+    <t>MAR</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>ESW_SIZE_M2</t>
+  </si>
+  <si>
+    <t>MWF_SIZE_M2</t>
+  </si>
+  <si>
+    <t>COVER_P</t>
+  </si>
+  <si>
+    <t>COVER_D</t>
+  </si>
+  <si>
+    <t>AVG_ESW_SIZE</t>
+  </si>
+  <si>
+    <t>ISFILL</t>
+  </si>
+  <si>
+    <t>MAR_D</t>
+  </si>
+  <si>
+    <t>MONTH</t>
+  </si>
+  <si>
+    <t>SIZ or Hydroshed</t>
+  </si>
+  <si>
+    <t>Shape ID</t>
+  </si>
+  <si>
+    <t>Time period</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Start of time period</t>
+  </si>
+  <si>
+    <t>End of time period</t>
+  </si>
+  <si>
+    <t># pixels in ESW for this shape</t>
+  </si>
+  <si>
+    <t># pixels in MWF for this shape</t>
+  </si>
+  <si>
+    <t>area of a single pixel</t>
+  </si>
+  <si>
+    <t>m2</t>
+  </si>
+  <si>
+    <t>mean annual rainfall for this shape and year</t>
+  </si>
+  <si>
+    <t>Size of ESW coverage for this shape and period</t>
+  </si>
+  <si>
+    <t>Size o MWF coverage for this shape</t>
+  </si>
+  <si>
+    <t>% of MWF covered by ESW in this period</t>
+  </si>
+  <si>
+    <t>anomaly of MWF coverage by ESW in this period, compared to mean</t>
+  </si>
+  <si>
+    <t>% difference from mean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean size of ESW </t>
+  </si>
+  <si>
+    <t>is there water at all in this time period?</t>
+  </si>
+  <si>
+    <t>boolean</t>
+  </si>
+  <si>
+    <t>anomaly of this shape's rainfall compared to mean for this shape</t>
+  </si>
+  <si>
+    <t>Month of data</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>Statistics on hydroshed and SIZ together, with monthly ESW as percent of MWF for statistical modeling and plotting</t>
+  </si>
+  <si>
+    <t>mardata</t>
+  </si>
+  <si>
+    <t>Mean annual rainfall - means and standard deviation for all of KAZA from 2019-2025, sorted by rainfall (mm)</t>
+  </si>
+  <si>
+    <t>mMAR</t>
+  </si>
+  <si>
+    <t>sdMAR</t>
+  </si>
+  <si>
+    <t>mean MAR across KAZA from 2019-2025</t>
+  </si>
+  <si>
+    <t>sd of MAR across KAZA from 2019-2025</t>
+  </si>
+  <si>
+    <t>year of data</t>
+  </si>
+  <si>
+    <t>/03_output/water_analysis.rdata</t>
   </si>
 </sst>
 </file>
@@ -435,7 +612,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -550,6 +727,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -595,7 +781,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -608,6 +794,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -994,7 +1181,7 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2"/>
       <c r="D1" s="3"/>
@@ -1025,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{675F3BD1-D2B9-134C-BD0B-8C3D6F403BE3}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
@@ -1034,18 +1221,18 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -1053,7 +1240,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1064,7 +1251,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>2</v>
@@ -1072,41 +1259,41 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8" s="4">
         <v>94</v>
@@ -1114,13 +1301,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D9" s="4">
         <v>100</v>
@@ -1128,13 +1315,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>17</v>
       </c>
       <c r="D10" s="4">
         <v>82</v>
@@ -1142,19 +1329,559 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="4">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B23" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="4">
+      <c r="C23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="4">
         <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1E2162F-5AEC-8143-B8B4-305B914ADF3B}">
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.33203125" customWidth="1"/>
+    <col min="2" max="2" width="58.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="3"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="5"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D36" s="4"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="2"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="4"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="4"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="4"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="2"/>
+      <c r="B40" s="2"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="2"/>
+      <c r="B43" s="2"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B44" s="2"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B45" s="2"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B46" s="2"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B47" s="2"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B48" s="2"/>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B49" s="2"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B50" s="2"/>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B51" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9107EEF2-C602-2D4E-B8A1-2D0FEF49D0AB}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{054E2CA6-F1EE-1D45-80C4-6FCC5C3B407F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>